<commit_message>
valora-demo: modelos Excel regenerados con Kd real ponderado por instrumento
Alicorp, Cía. de Minas Buenaventura, Cementos Pacasmayo e InRetail ahora usan
el Kd real por instrumento (deuda_financiera SMV) en vez del Kd implícito
(gastos financieros/deuda promedio), que estaba inflado en los 4 casos —
ej. Buenaventura pasó de 12.4% a 5.5%. Fuente: valora-ai commit b81117a
(kd_real.py, excel_modelo.py).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/valora-demo/modelos/alicorp-modelo.xlsx
+++ b/valora-demo/modelos/alicorp-modelo.xlsx
@@ -6008,11 +6008,11 @@
         </is>
       </c>
       <c r="C28" s="29" t="n">
-        <v>0.0991813253502055</v>
+        <v>0.0693</v>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>Default: |gastos financieros| / deuda financiera promedio (histórico)</t>
+          <t>Kd real ponderado por instrumento en PEN (deuda_financiera SMV, 100% saldo, 4/6 instrumentos) — ver kd_real.py</t>
         </is>
       </c>
     </row>

</xml_diff>